<commit_message>
v2.0 major upgrade: Phases 2-4
Phase 2 — Synergy + Ban Priority
- synergy_scores table, workbook sheet (38 known combos)
- Ban Priority section in draft results (threat = counter - vulnerability)
- Team Synergy display in Final Line-up modal

Phase 3 — Role Matrix + Teamfight Composition
- role_matrix integration in fight analysis (6x6 role matchup grid)
- teamfight_contribution column (-2 pure split-push to +2 wombo)
- Composition score (role diversity + tank/roamer + damage mix + TF)
- Role Advantage and Teamfight Potential bars in fight analysis

Phase 4 — Ban Simulator + Pick Urgency + Score Spread
- Ban Phase toggle with 5 ban slots, filters pool entirely
- Pick Early / Flexible urgency labels on result cards
- Score spread (min-max range) per candidate
</commit_message>
<xml_diff>
--- a/mobile_legends_heroes_updated.xlsx
+++ b/mobile_legends_heroes_updated.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CounterCalculator" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lookup" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LookupCalc" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synergy" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
@@ -159,7 +160,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -191,6 +192,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -477,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S134"/>
+  <dimension ref="A1:T134"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="5"/>
@@ -581,6 +585,11 @@
           <t>has_true_damage</t>
         </is>
       </c>
+      <c r="T1" s="23" t="inlineStr">
+        <is>
+          <t>teamfight_contribution</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" t="inlineStr">
@@ -658,6 +667,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T2" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" t="inlineStr">
@@ -740,6 +752,9 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="T3" s="23" t="n">
+        <v>-2</v>
+      </c>
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" t="inlineStr">
@@ -822,6 +837,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T4" s="23" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" t="inlineStr">
@@ -904,6 +922,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T5" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" t="inlineStr">
@@ -981,6 +1002,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T6" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" t="inlineStr">
@@ -1058,6 +1082,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T7" s="23" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" t="inlineStr">
@@ -1140,6 +1167,9 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="T8" s="23" t="n">
+        <v>-2</v>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" t="inlineStr">
@@ -1217,6 +1247,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T9" s="23" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" t="inlineStr">
@@ -1294,6 +1327,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T10" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" t="inlineStr">
@@ -1371,6 +1407,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T11" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" t="inlineStr">
@@ -1458,6 +1497,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T12" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" t="inlineStr">
@@ -1535,6 +1577,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T13" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" t="inlineStr">
@@ -1612,6 +1657,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T14" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" t="inlineStr">
@@ -1689,6 +1737,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T15" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" t="inlineStr">
@@ -1766,6 +1817,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T16" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" t="inlineStr">
@@ -1848,6 +1902,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T17" s="23" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" t="inlineStr">
@@ -1925,6 +1982,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T18" s="23" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" t="inlineStr">
@@ -2002,6 +2062,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T19" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" t="inlineStr">
@@ -2084,6 +2147,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T20" s="23" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" t="inlineStr">
@@ -2166,6 +2232,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T21" s="23" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" t="inlineStr">
@@ -2243,6 +2312,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T22" s="23" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" t="inlineStr">
@@ -2325,6 +2397,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T23" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" t="inlineStr">
@@ -2402,6 +2477,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T24" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="A25" t="inlineStr">
@@ -2484,6 +2562,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T25" s="23" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" t="inlineStr">
@@ -2561,6 +2642,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T26" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" t="inlineStr">
@@ -2643,6 +2727,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T27" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="A28" t="inlineStr">
@@ -2725,6 +2812,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T28" s="23" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="A29" t="inlineStr">
@@ -2807,6 +2897,9 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="T29" s="23" t="n">
+        <v>-2</v>
+      </c>
     </row>
     <row r="30" ht="15" customHeight="1">
       <c r="A30" t="inlineStr">
@@ -2884,6 +2977,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T30" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="31" ht="15" customHeight="1">
       <c r="A31" t="inlineStr">
@@ -2966,6 +3062,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T31" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="A32" t="inlineStr">
@@ -3043,6 +3142,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T32" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33" ht="15" customHeight="1">
       <c r="A33" t="inlineStr">
@@ -3125,6 +3227,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T33" s="23" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="34" ht="15" customHeight="1">
       <c r="A34" t="inlineStr">
@@ -3202,6 +3307,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T34" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35" ht="15" customHeight="1">
       <c r="A35" t="inlineStr">
@@ -3279,6 +3387,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T35" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="36" ht="15" customHeight="1">
       <c r="A36" t="inlineStr">
@@ -3366,6 +3477,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T36" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37" ht="15" customHeight="1">
       <c r="A37" t="inlineStr">
@@ -3443,6 +3557,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T37" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38" ht="15" customHeight="1">
       <c r="A38" t="inlineStr">
@@ -3520,6 +3637,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T38" s="23" t="n">
+        <v>-2</v>
+      </c>
     </row>
     <row r="39" ht="15" customHeight="1">
       <c r="A39" t="inlineStr">
@@ -3597,6 +3717,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T39" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="40" ht="15" customHeight="1">
       <c r="A40" t="inlineStr">
@@ -3679,6 +3802,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T40" s="23" t="n">
+        <v>-2</v>
+      </c>
     </row>
     <row r="41" ht="15" customHeight="1">
       <c r="A41" t="inlineStr">
@@ -3756,6 +3882,9 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="T41" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="A42" t="inlineStr">
@@ -3843,6 +3972,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T42" s="23" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="43" ht="15" customHeight="1">
       <c r="A43" t="inlineStr">
@@ -3930,6 +4062,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T43" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="44" ht="15" customHeight="1">
       <c r="A44" t="inlineStr">
@@ -4007,6 +4142,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T44" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="45" ht="15" customHeight="1">
       <c r="A45" t="inlineStr">
@@ -4089,6 +4227,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T45" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="46" ht="15" customHeight="1">
       <c r="A46" t="inlineStr">
@@ -4166,6 +4307,9 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="T46" s="23" t="n">
+        <v>-2</v>
+      </c>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="A47" t="inlineStr">
@@ -4243,6 +4387,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T47" s="23" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="48" ht="15" customHeight="1">
       <c r="A48" t="inlineStr">
@@ -4320,6 +4467,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T48" s="23" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="49" ht="15" customHeight="1">
       <c r="A49" t="inlineStr">
@@ -4397,6 +4547,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T49" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="50" ht="15" customHeight="1">
       <c r="A50" t="inlineStr">
@@ -4474,6 +4627,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T50" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="51" ht="15" customHeight="1">
       <c r="A51" t="inlineStr">
@@ -4551,6 +4707,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T51" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="52" ht="15" customHeight="1">
       <c r="A52" t="inlineStr">
@@ -4633,6 +4792,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T52" s="23" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="53" ht="15" customHeight="1">
       <c r="A53" t="inlineStr">
@@ -4710,6 +4872,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T53" s="23" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="54" ht="15" customHeight="1">
       <c r="A54" t="inlineStr">
@@ -4792,6 +4957,9 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="T54" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55" ht="15" customHeight="1">
       <c r="A55" t="inlineStr">
@@ -4874,6 +5042,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T55" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="56" ht="15" customHeight="1">
       <c r="A56" t="inlineStr">
@@ -4951,6 +5122,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T56" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="57" ht="15" customHeight="1">
       <c r="A57" t="inlineStr">
@@ -5033,6 +5207,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T57" s="23" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="58" ht="15" customHeight="1">
       <c r="A58" t="inlineStr">
@@ -5110,6 +5287,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T58" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="59" ht="15" customHeight="1">
       <c r="A59" t="inlineStr">
@@ -5192,6 +5372,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T59" s="23" t="n">
+        <v>-2</v>
+      </c>
     </row>
     <row r="60" ht="15" customHeight="1">
       <c r="A60" t="inlineStr">
@@ -5269,6 +5452,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T60" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="61" ht="15" customHeight="1">
       <c r="A61" t="inlineStr">
@@ -5346,6 +5532,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T61" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="62" ht="15" customHeight="1">
       <c r="A62" t="inlineStr">
@@ -5423,6 +5612,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T62" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="63" ht="15" customHeight="1">
       <c r="A63" t="inlineStr">
@@ -5505,6 +5697,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T63" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="64" ht="15" customHeight="1">
       <c r="A64" t="inlineStr">
@@ -5592,6 +5787,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T64" s="23" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="65" ht="15" customHeight="1">
       <c r="A65" t="inlineStr">
@@ -5669,6 +5867,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T65" s="23" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="66" ht="15" customHeight="1">
       <c r="A66" t="inlineStr">
@@ -5746,6 +5947,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T66" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="67" ht="15" customHeight="1">
       <c r="A67" t="inlineStr">
@@ -5823,6 +6027,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T67" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="68" ht="15" customHeight="1">
       <c r="A68" t="inlineStr">
@@ -5900,6 +6107,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T68" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="69" ht="15" customHeight="1">
       <c r="A69" t="inlineStr">
@@ -5977,6 +6187,9 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="T69" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="70" ht="15" customHeight="1">
       <c r="A70" t="inlineStr">
@@ -6054,6 +6267,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T70" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="71" ht="15" customHeight="1">
       <c r="A71" t="inlineStr">
@@ -6131,6 +6347,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T71" s="23" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="72" ht="15" customHeight="1">
       <c r="A72" t="inlineStr">
@@ -6218,6 +6437,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T72" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="73" ht="15" customHeight="1">
       <c r="A73" t="inlineStr">
@@ -6295,6 +6517,9 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="T73" s="23" t="n">
+        <v>-2</v>
+      </c>
     </row>
     <row r="74" ht="15" customHeight="1">
       <c r="A74" t="inlineStr">
@@ -6377,6 +6602,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T74" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="75" ht="15" customHeight="1">
       <c r="A75" t="inlineStr">
@@ -6459,6 +6687,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T75" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="76" ht="15" customHeight="1">
       <c r="A76" t="inlineStr">
@@ -6541,6 +6772,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T76" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="77" ht="15" customHeight="1">
       <c r="A77" t="inlineStr">
@@ -6628,6 +6862,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T77" s="23" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="78" ht="15" customHeight="1">
       <c r="A78" t="inlineStr">
@@ -6710,6 +6947,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T78" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="79" ht="15" customHeight="1">
       <c r="A79" t="inlineStr">
@@ -6787,6 +7027,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T79" s="23" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="80" ht="15" customHeight="1">
       <c r="A80" t="inlineStr">
@@ -6864,6 +7107,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T80" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="81" ht="15" customHeight="1">
       <c r="A81" t="inlineStr">
@@ -6941,6 +7187,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T81" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="82" ht="15" customHeight="1">
       <c r="A82" t="inlineStr">
@@ -7018,6 +7267,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T82" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="83" ht="15" customHeight="1">
       <c r="A83" t="inlineStr">
@@ -7100,6 +7352,9 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="T83" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="84" ht="15" customHeight="1">
       <c r="A84" t="inlineStr">
@@ -7177,6 +7432,9 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="T84" s="23" t="n">
+        <v>-2</v>
+      </c>
     </row>
     <row r="85" ht="15" customHeight="1">
       <c r="A85" t="inlineStr">
@@ -7254,6 +7512,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T85" s="23" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="86" ht="15" customHeight="1">
       <c r="A86" t="inlineStr">
@@ -7336,6 +7597,9 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="T86" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87" ht="15" customHeight="1">
       <c r="A87" t="inlineStr">
@@ -7413,6 +7677,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T87" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="88" ht="15" customHeight="1">
       <c r="A88" t="inlineStr">
@@ -7495,6 +7762,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T88" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="89" ht="15" customHeight="1">
       <c r="A89" t="inlineStr">
@@ -7577,6 +7847,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T89" s="23" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="90" ht="15" customHeight="1">
       <c r="A90" t="inlineStr">
@@ -7654,6 +7927,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T90" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="91" ht="15" customHeight="1">
       <c r="A91" t="inlineStr">
@@ -7731,6 +8007,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T91" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="92" ht="15" customHeight="1">
       <c r="A92" t="inlineStr">
@@ -7808,6 +8087,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T92" s="23" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="93" ht="15" customHeight="1">
       <c r="A93" t="inlineStr">
@@ -7890,6 +8172,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T93" s="23" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="94" ht="15" customHeight="1">
       <c r="A94" t="inlineStr">
@@ -7967,6 +8252,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T94" s="23" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="95" ht="15" customHeight="1">
       <c r="A95" t="inlineStr">
@@ -8049,6 +8337,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T95" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="96" ht="15" customHeight="1">
       <c r="A96" t="inlineStr">
@@ -8126,6 +8417,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T96" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="97" ht="15" customHeight="1">
       <c r="A97" t="inlineStr">
@@ -8203,6 +8497,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T97" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="98" ht="15" customHeight="1">
       <c r="A98" t="inlineStr">
@@ -8285,6 +8582,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T98" s="23" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="99" ht="15" customHeight="1">
       <c r="A99" t="inlineStr">
@@ -8367,6 +8667,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T99" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="100" ht="15" customHeight="1">
       <c r="A100" t="inlineStr">
@@ -8449,6 +8752,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T100" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101" ht="15" customHeight="1">
       <c r="A101" t="inlineStr">
@@ -8526,6 +8832,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T101" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="102" ht="15" customHeight="1">
       <c r="A102" t="inlineStr">
@@ -8603,6 +8912,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T102" s="23" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="103" ht="15" customHeight="1">
       <c r="A103" t="inlineStr">
@@ -8685,6 +8997,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T103" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="104" ht="15" customHeight="1">
       <c r="A104" t="inlineStr">
@@ -8767,6 +9082,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T104" s="23" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="105" ht="15" customHeight="1">
       <c r="A105" t="inlineStr">
@@ -8849,6 +9167,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T105" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="106" ht="15" customHeight="1">
       <c r="A106" t="inlineStr">
@@ -8926,6 +9247,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T106" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="107" ht="15" customHeight="1">
       <c r="A107" t="inlineStr">
@@ -9003,6 +9327,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T107" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="108" ht="15" customHeight="1">
       <c r="A108" t="inlineStr">
@@ -9080,6 +9407,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T108" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="109" ht="15" customHeight="1">
       <c r="A109" t="inlineStr">
@@ -9157,6 +9487,9 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="T109" s="23" t="n">
+        <v>-2</v>
+      </c>
     </row>
     <row r="110" ht="15" customHeight="1">
       <c r="A110" t="inlineStr">
@@ -9234,6 +9567,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T110" s="23" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="111" ht="15" customHeight="1">
       <c r="A111" t="inlineStr">
@@ -9311,6 +9647,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T111" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="112" ht="15" customHeight="1">
       <c r="A112" t="inlineStr">
@@ -9398,6 +9737,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T112" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="113" ht="15" customHeight="1">
       <c r="A113" t="inlineStr">
@@ -9475,6 +9817,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T113" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="114" ht="15" customHeight="1">
       <c r="A114" t="inlineStr">
@@ -9562,6 +9907,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T114" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="115" ht="15" customHeight="1">
       <c r="A115" t="inlineStr">
@@ -9639,6 +9987,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T115" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="116" ht="15" customHeight="1">
       <c r="A116" t="inlineStr">
@@ -9716,6 +10067,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T116" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="117" ht="15" customHeight="1">
       <c r="A117" t="inlineStr">
@@ -9803,6 +10157,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T117" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="118" ht="15" customHeight="1">
       <c r="A118" t="inlineStr">
@@ -9885,6 +10242,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T118" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="119" ht="15" customHeight="1">
       <c r="A119" t="inlineStr">
@@ -9962,6 +10322,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T119" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="120" ht="15" customHeight="1">
       <c r="A120" t="inlineStr">
@@ -10039,6 +10402,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T120" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="121" ht="15" customHeight="1">
       <c r="A121" t="inlineStr">
@@ -10121,6 +10487,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T121" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="122" ht="15" customHeight="1">
       <c r="A122" t="inlineStr">
@@ -10198,6 +10567,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T122" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="123" ht="15" customHeight="1">
       <c r="A123" t="inlineStr">
@@ -10275,6 +10647,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T123" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="124" ht="15" customHeight="1">
       <c r="A124" t="inlineStr">
@@ -10352,6 +10727,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T124" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="125" ht="15" customHeight="1">
       <c r="A125" t="inlineStr">
@@ -10434,6 +10812,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T125" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="126" ht="15" customHeight="1">
       <c r="A126" t="inlineStr">
@@ -10511,6 +10892,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T126" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="127" ht="15" customHeight="1">
       <c r="A127" t="inlineStr">
@@ -10593,6 +10977,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T127" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="128" ht="15" customHeight="1">
       <c r="A128" t="inlineStr">
@@ -10675,6 +11062,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T128" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="129" ht="15" customHeight="1">
       <c r="A129" t="inlineStr">
@@ -10757,6 +11147,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T129" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="130" ht="15" customHeight="1">
       <c r="A130" t="inlineStr">
@@ -10834,6 +11227,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T130" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="131" ht="15" customHeight="1">
       <c r="A131" t="inlineStr">
@@ -10911,6 +11307,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T131" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="132" ht="15" customHeight="1">
       <c r="A132" t="inlineStr">
@@ -10993,6 +11392,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T132" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="133" ht="15" customHeight="1">
       <c r="A133" t="inlineStr">
@@ -11070,6 +11472,9 @@
           <t>No</t>
         </is>
       </c>
+      <c r="T133" s="23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="134" ht="15" customHeight="1">
       <c r="A134" t="inlineStr">
@@ -11146,6 +11551,9 @@
         <is>
           <t>No</t>
         </is>
+      </c>
+      <c r="T134" s="23" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -44088,4 +44496,806 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D39"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="22" t="inlineStr">
+        <is>
+          <t>hero_a</t>
+        </is>
+      </c>
+      <c r="B1" s="22" t="inlineStr">
+        <is>
+          <t>hero_b</t>
+        </is>
+      </c>
+      <c r="C1" s="22" t="inlineStr">
+        <is>
+          <t>synergy</t>
+        </is>
+      </c>
+      <c r="D1" s="22" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="23" t="inlineStr">
+        <is>
+          <t>Johnson</t>
+        </is>
+      </c>
+      <c r="B2" s="23" t="inlineStr">
+        <is>
+          <t>Odette</t>
+        </is>
+      </c>
+      <c r="C2" s="23" t="n">
+        <v>18</v>
+      </c>
+      <c r="D2" s="24" t="inlineStr">
+        <is>
+          <t>Classic drive-by ult combo — Odette rides Johnson for a mobile nuke</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="23" t="inlineStr">
+        <is>
+          <t>Faramis</t>
+        </is>
+      </c>
+      <c r="B3" s="23" t="inlineStr">
+        <is>
+          <t>Pharsa</t>
+        </is>
+      </c>
+      <c r="C3" s="23" t="n">
+        <v>15</v>
+      </c>
+      <c r="D3" s="24" t="inlineStr">
+        <is>
+          <t>Resurrect lets Pharsa play hyper-aggressive, revive + full AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="23" t="inlineStr">
+        <is>
+          <t>Faramis</t>
+        </is>
+      </c>
+      <c r="B4" s="23" t="inlineStr">
+        <is>
+          <t>Yve</t>
+        </is>
+      </c>
+      <c r="C4" s="23" t="n">
+        <v>15</v>
+      </c>
+      <c r="D4" s="24" t="inlineStr">
+        <is>
+          <t>Same as Pharsa — Yve zone control with revive safety net</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="23" t="inlineStr">
+        <is>
+          <t>Tigreal</t>
+        </is>
+      </c>
+      <c r="B5" s="23" t="inlineStr">
+        <is>
+          <t>Pharsa</t>
+        </is>
+      </c>
+      <c r="C5" s="23" t="n">
+        <v>12</v>
+      </c>
+      <c r="D5" s="24" t="inlineStr">
+        <is>
+          <t>Tigreal setup into Pharsa raining death = teamfight wipe</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="23" t="inlineStr">
+        <is>
+          <t>Atlas</t>
+        </is>
+      </c>
+      <c r="B6" s="23" t="inlineStr">
+        <is>
+          <t>Pharsa</t>
+        </is>
+      </c>
+      <c r="C6" s="23" t="n">
+        <v>12</v>
+      </c>
+      <c r="D6" s="24" t="inlineStr">
+        <is>
+          <t>Fatal Links into Pharsa meteors = guaranteed full combo</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="23" t="inlineStr">
+        <is>
+          <t>Atlas</t>
+        </is>
+      </c>
+      <c r="B7" s="23" t="inlineStr">
+        <is>
+          <t>Odette</t>
+        </is>
+      </c>
+      <c r="C7" s="23" t="n">
+        <v>12</v>
+      </c>
+      <c r="D7" s="24" t="inlineStr">
+        <is>
+          <t>Fatal Links + Blue Nova = multi-man stun into full channel</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="23" t="inlineStr">
+        <is>
+          <t>Tigreal</t>
+        </is>
+      </c>
+      <c r="B8" s="23" t="inlineStr">
+        <is>
+          <t>Odette</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="D8" s="24" t="inlineStr">
+        <is>
+          <t>Implosion setup into Odette ult</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="23" t="inlineStr">
+        <is>
+          <t>Lolita</t>
+        </is>
+      </c>
+      <c r="B9" s="23" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C9" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="D9" s="24" t="inlineStr">
+        <is>
+          <t>Shield blocks enemy projectiles while Claude shreds</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="23" t="inlineStr">
+        <is>
+          <t>Lolita</t>
+        </is>
+      </c>
+      <c r="B10" s="23" t="inlineStr">
+        <is>
+          <t>Chang'e</t>
+        </is>
+      </c>
+      <c r="C10" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="D10" s="24" t="inlineStr">
+        <is>
+          <t>Same mechanic — Chang'e poke/ult behind Lolita shield</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="23" t="inlineStr">
+        <is>
+          <t>Mathilda</t>
+        </is>
+      </c>
+      <c r="B11" s="23" t="inlineStr">
+        <is>
+          <t>Lancelot</t>
+        </is>
+      </c>
+      <c r="C11" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="D11" s="24" t="inlineStr">
+        <is>
+          <t>Guiding Wind lets Lancelot dive deeper + reset more safely</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="23" t="inlineStr">
+        <is>
+          <t>Mathilda</t>
+        </is>
+      </c>
+      <c r="B12" s="23" t="inlineStr">
+        <is>
+          <t>Hayabusa</t>
+        </is>
+      </c>
+      <c r="C12" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="D12" s="24" t="inlineStr">
+        <is>
+          <t>Same — Mathilda ult follows Haya shadow for chain dives</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="23" t="inlineStr">
+        <is>
+          <t>Mathilda</t>
+        </is>
+      </c>
+      <c r="B13" s="23" t="inlineStr">
+        <is>
+          <t>Ling</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="D13" s="24" t="inlineStr">
+        <is>
+          <t>Ling + Mathilda = unmatched backline access</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="23" t="inlineStr">
+        <is>
+          <t>Mathilda</t>
+        </is>
+      </c>
+      <c r="B14" s="23" t="inlineStr">
+        <is>
+          <t>Alucard</t>
+        </is>
+      </c>
+      <c r="C14" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D14" s="24" t="inlineStr">
+        <is>
+          <t>Dive + lifesteal synergy, Alucard gets in and stays in</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="23" t="inlineStr">
+        <is>
+          <t>Kaja</t>
+        </is>
+      </c>
+      <c r="B15" s="23" t="inlineStr">
+        <is>
+          <t>Hayabusa</t>
+        </is>
+      </c>
+      <c r="C15" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="D15" s="24" t="inlineStr">
+        <is>
+          <t>Kaja suppress + Hayabusa full Ougi = guaranteed kill</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="23" t="inlineStr">
+        <is>
+          <t>Kaja</t>
+        </is>
+      </c>
+      <c r="B16" s="23" t="inlineStr">
+        <is>
+          <t>Aldous</t>
+        </is>
+      </c>
+      <c r="C16" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="D16" s="24" t="inlineStr">
+        <is>
+          <t>Kaja suppress + Aldous ult = uncontested punch</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="23" t="inlineStr">
+        <is>
+          <t>Kaja</t>
+        </is>
+      </c>
+      <c r="B17" s="23" t="inlineStr">
+        <is>
+          <t>Helcurt</t>
+        </is>
+      </c>
+      <c r="C17" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="D17" s="24" t="inlineStr">
+        <is>
+          <t>Suppress + silence = no escape, no counterplay</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="23" t="inlineStr">
+        <is>
+          <t>Chou</t>
+        </is>
+      </c>
+      <c r="B18" s="23" t="inlineStr">
+        <is>
+          <t>Lancelot</t>
+        </is>
+      </c>
+      <c r="C18" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D18" s="24" t="inlineStr">
+        <is>
+          <t>Chou setup knock-up into Lancelot reset chain</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="23" t="inlineStr">
+        <is>
+          <t>Angela</t>
+        </is>
+      </c>
+      <c r="B19" s="23" t="inlineStr">
+        <is>
+          <t>Esmeralda</t>
+        </is>
+      </c>
+      <c r="C19" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D19" s="24" t="inlineStr">
+        <is>
+          <t>Angela link + shield lets Esme dive without dying</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="23" t="inlineStr">
+        <is>
+          <t>Angela</t>
+        </is>
+      </c>
+      <c r="B20" s="23" t="inlineStr">
+        <is>
+          <t>Thamuz</t>
+        </is>
+      </c>
+      <c r="C20" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="D20" s="24" t="inlineStr">
+        <is>
+          <t>Thamuz becomes unkillable with Angela rot, wins manfights</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="23" t="inlineStr">
+        <is>
+          <t>Angela</t>
+        </is>
+      </c>
+      <c r="B21" s="23" t="inlineStr">
+        <is>
+          <t>Uranus</t>
+        </is>
+      </c>
+      <c r="C21" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D21" s="24" t="inlineStr">
+        <is>
+          <t>Already durable Uranus becomes immortal with Angela</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="23" t="inlineStr">
+        <is>
+          <t>Angela</t>
+        </is>
+      </c>
+      <c r="B22" s="23" t="inlineStr">
+        <is>
+          <t>Terizla</t>
+        </is>
+      </c>
+      <c r="C22" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D22" s="24" t="inlineStr">
+        <is>
+          <t>Terizla slow + Angela speed = sticky frontliner</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="23" t="inlineStr">
+        <is>
+          <t>Estes</t>
+        </is>
+      </c>
+      <c r="B23" s="23" t="inlineStr">
+        <is>
+          <t>Belerick</t>
+        </is>
+      </c>
+      <c r="C23" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D23" s="24" t="inlineStr">
+        <is>
+          <t>Estes chain heal + Belerick taunt = never-dying frontline</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="23" t="inlineStr">
+        <is>
+          <t>Estes</t>
+        </is>
+      </c>
+      <c r="B24" s="23" t="inlineStr">
+        <is>
+          <t>Uranus</t>
+        </is>
+      </c>
+      <c r="C24" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D24" s="24" t="inlineStr">
+        <is>
+          <t>Same — Uranus with Estes heals is nearly impossible to burst</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="23" t="inlineStr">
+        <is>
+          <t>Estes</t>
+        </is>
+      </c>
+      <c r="B25" s="23" t="inlineStr">
+        <is>
+          <t>Esmeralda</t>
+        </is>
+      </c>
+      <c r="C25" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D25" s="24" t="inlineStr">
+        <is>
+          <t>Esme + Estes = infinite shield rotation</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="23" t="inlineStr">
+        <is>
+          <t>Franco</t>
+        </is>
+      </c>
+      <c r="B26" s="23" t="inlineStr">
+        <is>
+          <t>Aldous</t>
+        </is>
+      </c>
+      <c r="C26" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="D26" s="24" t="inlineStr">
+        <is>
+          <t>Hook + Aldous ult = guaranteed kill on any hooked target</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="23" t="inlineStr">
+        <is>
+          <t>Franco</t>
+        </is>
+      </c>
+      <c r="B27" s="23" t="inlineStr">
+        <is>
+          <t>Selena</t>
+        </is>
+      </c>
+      <c r="C27" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="D27" s="24" t="inlineStr">
+        <is>
+          <t>Hook + Selena arrow = infinite chain CC</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="23" t="inlineStr">
+        <is>
+          <t>Selena</t>
+        </is>
+      </c>
+      <c r="B28" s="23" t="inlineStr">
+        <is>
+          <t>Helcurt</t>
+        </is>
+      </c>
+      <c r="C28" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D28" s="24" t="inlineStr">
+        <is>
+          <t>Selena stun + Helcurt silence = no escape window</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="23" t="inlineStr">
+        <is>
+          <t>Selena</t>
+        </is>
+      </c>
+      <c r="B29" s="23" t="inlineStr">
+        <is>
+          <t>Hayabusa</t>
+        </is>
+      </c>
+      <c r="C29" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D29" s="24" t="inlineStr">
+        <is>
+          <t>Selena arrow into Haya Ougi = dead before stun ends</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="23" t="inlineStr">
+        <is>
+          <t>Helcurt</t>
+        </is>
+      </c>
+      <c r="B30" s="23" t="inlineStr">
+        <is>
+          <t>Atlas</t>
+        </is>
+      </c>
+      <c r="C30" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="D30" s="24" t="inlineStr">
+        <is>
+          <t>Global silence prevents all counterplay vs Atlas engage</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="23" t="inlineStr">
+        <is>
+          <t>Helcurt</t>
+        </is>
+      </c>
+      <c r="B31" s="23" t="inlineStr">
+        <is>
+          <t>Tigreal</t>
+        </is>
+      </c>
+      <c r="C31" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="D31" s="24" t="inlineStr">
+        <is>
+          <t>Same — silence + Implosion = no skills to escape</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="23" t="inlineStr">
+        <is>
+          <t>Helcurt</t>
+        </is>
+      </c>
+      <c r="B32" s="23" t="inlineStr">
+        <is>
+          <t>Pharsa</t>
+        </is>
+      </c>
+      <c r="C32" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="D32" s="24" t="inlineStr">
+        <is>
+          <t>Silence into Pharsa rain = no skills to dodge</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="23" t="inlineStr">
+        <is>
+          <t>Helcurt</t>
+        </is>
+      </c>
+      <c r="B33" s="23" t="inlineStr">
+        <is>
+          <t>Kaja</t>
+        </is>
+      </c>
+      <c r="C33" s="23" t="n">
+        <v>12</v>
+      </c>
+      <c r="D33" s="24" t="inlineStr">
+        <is>
+          <t>Silence + suppress = absolute lockdown, no counterplay</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="23" t="inlineStr">
+        <is>
+          <t>Johnson</t>
+        </is>
+      </c>
+      <c r="B34" s="23" t="inlineStr">
+        <is>
+          <t>Faramis</t>
+        </is>
+      </c>
+      <c r="C34" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="D34" s="24" t="inlineStr">
+        <is>
+          <t>Taxi(Johnson) + revive(Faramis) = supreme rotation threat</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="23" t="inlineStr">
+        <is>
+          <t>Rafaela</t>
+        </is>
+      </c>
+      <c r="B35" s="23" t="inlineStr">
+        <is>
+          <t>Aldous</t>
+        </is>
+      </c>
+      <c r="C35" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="D35" s="24" t="inlineStr">
+        <is>
+          <t>Rafaela speed boost + Aldous ult = global pressure</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="23" t="inlineStr">
+        <is>
+          <t>Rafaela</t>
+        </is>
+      </c>
+      <c r="B36" s="23" t="inlineStr">
+        <is>
+          <t>Lunox</t>
+        </is>
+      </c>
+      <c r="C36" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="D36" s="24" t="inlineStr">
+        <is>
+          <t>Speed + sustain helps Lunox position for chaos ult</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="23" t="inlineStr">
+        <is>
+          <t>Diggie</t>
+        </is>
+      </c>
+      <c r="B37" s="23" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C37" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D37" s="24" t="inlineStr">
+        <is>
+          <t>Diggie egg + purify saves Claude from dive attempts</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="23" t="inlineStr">
+        <is>
+          <t>Diggie</t>
+        </is>
+      </c>
+      <c r="B38" s="23" t="inlineStr">
+        <is>
+          <t>Beatrix</t>
+        </is>
+      </c>
+      <c r="C38" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D38" s="24" t="inlineStr">
+        <is>
+          <t>Same — Diggie disengages divers for Beatrix</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="23" t="inlineStr">
+        <is>
+          <t>Diggie</t>
+        </is>
+      </c>
+      <c r="B39" s="23" t="inlineStr">
+        <is>
+          <t>Lunox</t>
+        </is>
+      </c>
+      <c r="C39" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D39" s="24" t="inlineStr">
+        <is>
+          <t>Diggie ult lets Lunox play aggressive, immune to CC</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
audit and fix hard_counter_rules: deduplicate Khufra entries, document conventions
Structural issues found and fixed:
- Khufra had duplicate (Tag|Dash/Blink, Tag|High Mobility) rows causing
  double-stacking in hard_counter_bonus() (21/-23 and 25/-27 instead of
  10/-10 and 14/-14). Older asymmetric entries cleared from Excel.
- 3 stale lowercase-variant rows in Supabase (angela, harley, saber)
  deleted — would double-stack after _norm() normalization.
- Phoveus mobility tags verified safe: no hero carries multiple
  mobility tags, so his three rules are mutually exclusive per defender.
- Baxia cross-condition stacking documented: 16 heroes match 2+
  conditions; stacked totals (40-49) are proportionate.
- Applied 100 rules through migrate and recompute (17556 rows).
</commit_message>
<xml_diff>
--- a/mobile_legends_heroes_updated.xlsx
+++ b/mobile_legends_heroes_updated.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -115,6 +115,11 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00CC4444"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -160,7 +165,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -196,6 +201,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -11571,7 +11577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W1190"/>
+  <dimension ref="A1:W1191"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -12180,32 +12186,12 @@
       </c>
     </row>
     <row r="34" ht="15" customHeight="1">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>Khufra</t>
-        </is>
-      </c>
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>Tag</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="inlineStr">
-        <is>
-          <t>Dash/Blink</t>
-        </is>
-      </c>
-      <c r="D34" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="E34" s="4" t="n">
-        <v>-13</v>
-      </c>
-      <c r="F34" s="3" t="inlineStr">
-        <is>
-          <t>Bouncing Ball cancels dashes/blinks mid-animation, hard-locking mobility divers.</t>
-        </is>
-      </c>
+      <c r="A34" s="4" t="n"/>
+      <c r="B34" s="4" t="n"/>
+      <c r="C34" s="4" t="n"/>
+      <c r="D34" s="4" t="n"/>
+      <c r="E34" s="4" t="n"/>
+      <c r="F34" s="3" t="n"/>
       <c r="J34" t="inlineStr">
         <is>
           <t>Energy</t>
@@ -12213,32 +12199,12 @@
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>Khufra</t>
-        </is>
-      </c>
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>Tag</t>
-        </is>
-      </c>
-      <c r="C35" s="4" t="inlineStr">
-        <is>
-          <t>High Mobility</t>
-        </is>
-      </c>
-      <c r="D35" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="E35" s="4" t="n">
-        <v>-13</v>
-      </c>
-      <c r="F35" s="3" t="inlineStr">
-        <is>
-          <t>Sturdiness plus Charging Roar punish sustained-mobility assassins.</t>
-        </is>
-      </c>
+      <c r="A35" s="4" t="n"/>
+      <c r="B35" s="4" t="n"/>
+      <c r="C35" s="4" t="n"/>
+      <c r="D35" s="4" t="n"/>
+      <c r="E35" s="4" t="n"/>
+      <c r="F35" s="3" t="n"/>
       <c r="J35" t="inlineStr">
         <is>
           <t>None</t>
@@ -27435,6 +27401,13 @@
       <c r="E1190">
         <f>A1190&amp;"|"&amp;B1190</f>
         <v/>
+      </c>
+    </row>
+    <row r="1191">
+      <c r="A1191" s="25" t="inlineStr">
+        <is>
+          <t>CONVENTION: Hard counter rules default to symmetric values (bonus_to_attacker = -penalty_to_defender). Asymmetric values are allowed when a specific matchup requires the attacker to benefit more (or less) than the defender is penalized, but this should be the exception, not the rule.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix fight mode composition penalty
- Add compositionPenalty() — subtracts from team totals for role
  stacking, missing critical roles, and damage homogeneity
- 5× same role: -90, 4×: -55, 3×: -30; no roamer: -25;
  no ranged DPS: -20; all same damage: -12
- Display penalty breakdown in fight verdict bar
- Add narrative sentence in Deciding Factors when penalty ≥20
- Fix RLS: disable row-level security on synergy_scores & role_matrix
- Add Lolita + Hanabi synergy (value 10) to Excel and migrate
</commit_message>
<xml_diff>
--- a/mobile_legends_heroes_updated.xlsx
+++ b/mobile_legends_heroes_updated.xlsx
@@ -165,7 +165,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -202,6 +202,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="bottom" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -44477,7 +44480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -44689,22 +44692,22 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="23" t="inlineStr">
-        <is>
-          <t>Mathilda</t>
-        </is>
-      </c>
-      <c r="B11" s="23" t="inlineStr">
-        <is>
-          <t>Lancelot</t>
-        </is>
-      </c>
-      <c r="C11" s="23" t="n">
+      <c r="A11" s="26" t="inlineStr">
+        <is>
+          <t>Lolita</t>
+        </is>
+      </c>
+      <c r="B11" s="26" t="inlineStr">
+        <is>
+          <t>Hanabi</t>
+        </is>
+      </c>
+      <c r="C11" s="26" t="n">
         <v>10</v>
       </c>
-      <c r="D11" s="24" t="inlineStr">
-        <is>
-          <t>Guiding Wind lets Lancelot dive deeper + reset more safely</t>
+      <c r="D11" s="26" t="inlineStr">
+        <is>
+          <t>Lolita shield blocks projectiles while Hanabi bouncing attacks punish clumped enemies</t>
         </is>
       </c>
     </row>
@@ -44716,7 +44719,7 @@
       </c>
       <c r="B12" s="23" t="inlineStr">
         <is>
-          <t>Hayabusa</t>
+          <t>Lancelot</t>
         </is>
       </c>
       <c r="C12" s="23" t="n">
@@ -44724,7 +44727,7 @@
       </c>
       <c r="D12" s="24" t="inlineStr">
         <is>
-          <t>Same — Mathilda ult follows Haya shadow for chain dives</t>
+          <t>Guiding Wind lets Lancelot dive deeper + reset more safely</t>
         </is>
       </c>
     </row>
@@ -44736,7 +44739,7 @@
       </c>
       <c r="B13" s="23" t="inlineStr">
         <is>
-          <t>Ling</t>
+          <t>Hayabusa</t>
         </is>
       </c>
       <c r="C13" s="23" t="n">
@@ -44744,7 +44747,7 @@
       </c>
       <c r="D13" s="24" t="inlineStr">
         <is>
-          <t>Ling + Mathilda = unmatched backline access</t>
+          <t>Same — Mathilda ult follows Haya shadow for chain dives</t>
         </is>
       </c>
     </row>
@@ -44756,35 +44759,35 @@
       </c>
       <c r="B14" s="23" t="inlineStr">
         <is>
-          <t>Alucard</t>
+          <t>Ling</t>
         </is>
       </c>
       <c r="C14" s="23" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D14" s="24" t="inlineStr">
         <is>
-          <t>Dive + lifesteal synergy, Alucard gets in and stays in</t>
+          <t>Ling + Mathilda = unmatched backline access</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="23" t="inlineStr">
         <is>
-          <t>Kaja</t>
+          <t>Mathilda</t>
         </is>
       </c>
       <c r="B15" s="23" t="inlineStr">
         <is>
-          <t>Hayabusa</t>
+          <t>Alucard</t>
         </is>
       </c>
       <c r="C15" s="23" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D15" s="24" t="inlineStr">
         <is>
-          <t>Kaja suppress + Hayabusa full Ougi = guaranteed kill</t>
+          <t>Dive + lifesteal synergy, Alucard gets in and stays in</t>
         </is>
       </c>
     </row>
@@ -44796,7 +44799,7 @@
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>Aldous</t>
+          <t>Hayabusa</t>
         </is>
       </c>
       <c r="C16" s="23" t="n">
@@ -44804,7 +44807,7 @@
       </c>
       <c r="D16" s="24" t="inlineStr">
         <is>
-          <t>Kaja suppress + Aldous ult = uncontested punch</t>
+          <t>Kaja suppress + Hayabusa full Ougi = guaranteed kill</t>
         </is>
       </c>
     </row>
@@ -44816,7 +44819,7 @@
       </c>
       <c r="B17" s="23" t="inlineStr">
         <is>
-          <t>Helcurt</t>
+          <t>Aldous</t>
         </is>
       </c>
       <c r="C17" s="23" t="n">
@@ -44824,39 +44827,39 @@
       </c>
       <c r="D17" s="24" t="inlineStr">
         <is>
-          <t>Suppress + silence = no escape, no counterplay</t>
+          <t>Kaja suppress + Aldous ult = uncontested punch</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="23" t="inlineStr">
         <is>
-          <t>Chou</t>
+          <t>Kaja</t>
         </is>
       </c>
       <c r="B18" s="23" t="inlineStr">
         <is>
-          <t>Lancelot</t>
+          <t>Helcurt</t>
         </is>
       </c>
       <c r="C18" s="23" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D18" s="24" t="inlineStr">
         <is>
-          <t>Chou setup knock-up into Lancelot reset chain</t>
+          <t>Suppress + silence = no escape, no counterplay</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="23" t="inlineStr">
         <is>
-          <t>Angela</t>
+          <t>Chou</t>
         </is>
       </c>
       <c r="B19" s="23" t="inlineStr">
         <is>
-          <t>Esmeralda</t>
+          <t>Lancelot</t>
         </is>
       </c>
       <c r="C19" s="23" t="n">
@@ -44864,7 +44867,7 @@
       </c>
       <c r="D19" s="24" t="inlineStr">
         <is>
-          <t>Angela link + shield lets Esme dive without dying</t>
+          <t>Chou setup knock-up into Lancelot reset chain</t>
         </is>
       </c>
     </row>
@@ -44876,15 +44879,15 @@
       </c>
       <c r="B20" s="23" t="inlineStr">
         <is>
-          <t>Thamuz</t>
+          <t>Esmeralda</t>
         </is>
       </c>
       <c r="C20" s="23" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D20" s="24" t="inlineStr">
         <is>
-          <t>Thamuz becomes unkillable with Angela rot, wins manfights</t>
+          <t>Angela link + shield lets Esme dive without dying</t>
         </is>
       </c>
     </row>
@@ -44896,15 +44899,15 @@
       </c>
       <c r="B21" s="23" t="inlineStr">
         <is>
-          <t>Uranus</t>
+          <t>Thamuz</t>
         </is>
       </c>
       <c r="C21" s="23" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D21" s="24" t="inlineStr">
         <is>
-          <t>Already durable Uranus becomes immortal with Angela</t>
+          <t>Thamuz becomes unkillable with Angela rot, wins manfights</t>
         </is>
       </c>
     </row>
@@ -44916,7 +44919,7 @@
       </c>
       <c r="B22" s="23" t="inlineStr">
         <is>
-          <t>Terizla</t>
+          <t>Uranus</t>
         </is>
       </c>
       <c r="C22" s="23" t="n">
@@ -44924,19 +44927,19 @@
       </c>
       <c r="D22" s="24" t="inlineStr">
         <is>
-          <t>Terizla slow + Angela speed = sticky frontliner</t>
+          <t>Already durable Uranus becomes immortal with Angela</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="23" t="inlineStr">
         <is>
-          <t>Estes</t>
+          <t>Angela</t>
         </is>
       </c>
       <c r="B23" s="23" t="inlineStr">
         <is>
-          <t>Belerick</t>
+          <t>Terizla</t>
         </is>
       </c>
       <c r="C23" s="23" t="n">
@@ -44944,7 +44947,7 @@
       </c>
       <c r="D23" s="24" t="inlineStr">
         <is>
-          <t>Estes chain heal + Belerick taunt = never-dying frontline</t>
+          <t>Terizla slow + Angela speed = sticky frontliner</t>
         </is>
       </c>
     </row>
@@ -44956,7 +44959,7 @@
       </c>
       <c r="B24" s="23" t="inlineStr">
         <is>
-          <t>Uranus</t>
+          <t>Belerick</t>
         </is>
       </c>
       <c r="C24" s="23" t="n">
@@ -44964,7 +44967,7 @@
       </c>
       <c r="D24" s="24" t="inlineStr">
         <is>
-          <t>Same — Uranus with Estes heals is nearly impossible to burst</t>
+          <t>Estes chain heal + Belerick taunt = never-dying frontline</t>
         </is>
       </c>
     </row>
@@ -44976,7 +44979,7 @@
       </c>
       <c r="B25" s="23" t="inlineStr">
         <is>
-          <t>Esmeralda</t>
+          <t>Uranus</t>
         </is>
       </c>
       <c r="C25" s="23" t="n">
@@ -44984,27 +44987,27 @@
       </c>
       <c r="D25" s="24" t="inlineStr">
         <is>
-          <t>Esme + Estes = infinite shield rotation</t>
+          <t>Same — Uranus with Estes heals is nearly impossible to burst</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="23" t="inlineStr">
         <is>
-          <t>Franco</t>
+          <t>Estes</t>
         </is>
       </c>
       <c r="B26" s="23" t="inlineStr">
         <is>
-          <t>Aldous</t>
+          <t>Esmeralda</t>
         </is>
       </c>
       <c r="C26" s="23" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D26" s="24" t="inlineStr">
         <is>
-          <t>Hook + Aldous ult = guaranteed kill on any hooked target</t>
+          <t>Esme + Estes = infinite shield rotation</t>
         </is>
       </c>
     </row>
@@ -45016,7 +45019,7 @@
       </c>
       <c r="B27" s="23" t="inlineStr">
         <is>
-          <t>Selena</t>
+          <t>Aldous</t>
         </is>
       </c>
       <c r="C27" s="23" t="n">
@@ -45024,27 +45027,27 @@
       </c>
       <c r="D27" s="24" t="inlineStr">
         <is>
-          <t>Hook + Selena arrow = infinite chain CC</t>
+          <t>Hook + Aldous ult = guaranteed kill on any hooked target</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="23" t="inlineStr">
         <is>
+          <t>Franco</t>
+        </is>
+      </c>
+      <c r="B28" s="23" t="inlineStr">
+        <is>
           <t>Selena</t>
         </is>
       </c>
-      <c r="B28" s="23" t="inlineStr">
-        <is>
-          <t>Helcurt</t>
-        </is>
-      </c>
       <c r="C28" s="23" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D28" s="24" t="inlineStr">
         <is>
-          <t>Selena stun + Helcurt silence = no escape window</t>
+          <t>Hook + Selena arrow = infinite chain CC</t>
         </is>
       </c>
     </row>
@@ -45056,7 +45059,7 @@
       </c>
       <c r="B29" s="23" t="inlineStr">
         <is>
-          <t>Hayabusa</t>
+          <t>Helcurt</t>
         </is>
       </c>
       <c r="C29" s="23" t="n">
@@ -45064,27 +45067,27 @@
       </c>
       <c r="D29" s="24" t="inlineStr">
         <is>
-          <t>Selena arrow into Haya Ougi = dead before stun ends</t>
+          <t>Selena stun + Helcurt silence = no escape window</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="23" t="inlineStr">
         <is>
-          <t>Helcurt</t>
+          <t>Selena</t>
         </is>
       </c>
       <c r="B30" s="23" t="inlineStr">
         <is>
-          <t>Atlas</t>
+          <t>Hayabusa</t>
         </is>
       </c>
       <c r="C30" s="23" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D30" s="24" t="inlineStr">
         <is>
-          <t>Global silence prevents all counterplay vs Atlas engage</t>
+          <t>Selena arrow into Haya Ougi = dead before stun ends</t>
         </is>
       </c>
     </row>
@@ -45096,7 +45099,7 @@
       </c>
       <c r="B31" s="23" t="inlineStr">
         <is>
-          <t>Tigreal</t>
+          <t>Atlas</t>
         </is>
       </c>
       <c r="C31" s="23" t="n">
@@ -45104,7 +45107,7 @@
       </c>
       <c r="D31" s="24" t="inlineStr">
         <is>
-          <t>Same — silence + Implosion = no skills to escape</t>
+          <t>Global silence prevents all counterplay vs Atlas engage</t>
         </is>
       </c>
     </row>
@@ -45116,7 +45119,7 @@
       </c>
       <c r="B32" s="23" t="inlineStr">
         <is>
-          <t>Pharsa</t>
+          <t>Tigreal</t>
         </is>
       </c>
       <c r="C32" s="23" t="n">
@@ -45124,7 +45127,7 @@
       </c>
       <c r="D32" s="24" t="inlineStr">
         <is>
-          <t>Silence into Pharsa rain = no skills to dodge</t>
+          <t>Same — silence + Implosion = no skills to escape</t>
         </is>
       </c>
     </row>
@@ -45136,47 +45139,47 @@
       </c>
       <c r="B33" s="23" t="inlineStr">
         <is>
-          <t>Kaja</t>
+          <t>Pharsa</t>
         </is>
       </c>
       <c r="C33" s="23" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D33" s="24" t="inlineStr">
         <is>
-          <t>Silence + suppress = absolute lockdown, no counterplay</t>
+          <t>Silence into Pharsa rain = no skills to dodge</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="23" t="inlineStr">
         <is>
-          <t>Johnson</t>
+          <t>Helcurt</t>
         </is>
       </c>
       <c r="B34" s="23" t="inlineStr">
         <is>
-          <t>Faramis</t>
+          <t>Kaja</t>
         </is>
       </c>
       <c r="C34" s="23" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D34" s="24" t="inlineStr">
         <is>
-          <t>Taxi(Johnson) + revive(Faramis) = supreme rotation threat</t>
+          <t>Silence + suppress = absolute lockdown, no counterplay</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="23" t="inlineStr">
         <is>
-          <t>Rafaela</t>
+          <t>Johnson</t>
         </is>
       </c>
       <c r="B35" s="23" t="inlineStr">
         <is>
-          <t>Aldous</t>
+          <t>Faramis</t>
         </is>
       </c>
       <c r="C35" s="23" t="n">
@@ -45184,7 +45187,7 @@
       </c>
       <c r="D35" s="24" t="inlineStr">
         <is>
-          <t>Rafaela speed boost + Aldous ult = global pressure</t>
+          <t>Taxi(Johnson) + revive(Faramis) = supreme rotation threat</t>
         </is>
       </c>
     </row>
@@ -45196,7 +45199,7 @@
       </c>
       <c r="B36" s="23" t="inlineStr">
         <is>
-          <t>Lunox</t>
+          <t>Aldous</t>
         </is>
       </c>
       <c r="C36" s="23" t="n">
@@ -45204,27 +45207,27 @@
       </c>
       <c r="D36" s="24" t="inlineStr">
         <is>
-          <t>Speed + sustain helps Lunox position for chaos ult</t>
+          <t>Rafaela speed boost + Aldous ult = global pressure</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="23" t="inlineStr">
         <is>
-          <t>Diggie</t>
+          <t>Rafaela</t>
         </is>
       </c>
       <c r="B37" s="23" t="inlineStr">
         <is>
-          <t>Claude</t>
+          <t>Lunox</t>
         </is>
       </c>
       <c r="C37" s="23" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D37" s="24" t="inlineStr">
         <is>
-          <t>Diggie egg + purify saves Claude from dive attempts</t>
+          <t>Speed + sustain helps Lunox position for chaos ult</t>
         </is>
       </c>
     </row>
@@ -45236,7 +45239,7 @@
       </c>
       <c r="B38" s="23" t="inlineStr">
         <is>
-          <t>Beatrix</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="C38" s="23" t="n">
@@ -45244,7 +45247,7 @@
       </c>
       <c r="D38" s="24" t="inlineStr">
         <is>
-          <t>Same — Diggie disengages divers for Beatrix</t>
+          <t>Diggie egg + purify saves Claude from dive attempts</t>
         </is>
       </c>
     </row>
@@ -45256,13 +45259,33 @@
       </c>
       <c r="B39" s="23" t="inlineStr">
         <is>
-          <t>Lunox</t>
+          <t>Beatrix</t>
         </is>
       </c>
       <c r="C39" s="23" t="n">
         <v>8</v>
       </c>
       <c r="D39" s="24" t="inlineStr">
+        <is>
+          <t>Same — Diggie disengages divers for Beatrix</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="23" t="inlineStr">
+        <is>
+          <t>Diggie</t>
+        </is>
+      </c>
+      <c r="B40" s="23" t="inlineStr">
+        <is>
+          <t>Lunox</t>
+        </is>
+      </c>
+      <c r="C40" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D40" s="24" t="inlineStr">
         <is>
           <t>Diggie ult lets Lunox play aggressive, immune to CC</t>
         </is>

</xml_diff>

<commit_message>
add 3 synergies: Bruno+Diggie, Ixia+Diggie, Johnson+Arlott
</commit_message>
<xml_diff>
--- a/mobile_legends_heroes_updated.xlsx
+++ b/mobile_legends_heroes_updated.xlsx
@@ -44537,7 +44537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" style="21" min="1" max="2"/>
@@ -45347,6 +45347,66 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Bruno</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Diggie</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>8</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Diggie egg/shield protects Bruno from dive; Bruno burst punishes enemies who target Diggie</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Ixia</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Diggie</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>8</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Diggie egg shields Ixia from burst; Ixia AoE punishes enemies diving for Diggie</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Johnson</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Arlott</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>12</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Johnson Drive rides Arlott for mobile ganks; Arlott blink extends Johnson Drive range</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>